<commit_message>
Updated biomarker analysis (nb + results).
</commit_message>
<xml_diff>
--- a/results/cluster_analysis/feature_selection_ABESS.xlsx
+++ b/results/cluster_analysis/feature_selection_ABESS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos Paja Suarez\imoc_pdac\results\cluster_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B2C3F10-DE1C-49E4-8C19-9A8119E39B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C617998-99FD-4538-8EA1-14C7770D1770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{5BF63DF1-7A44-450C-B389-D944A32FFCF8}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{5BF63DF1-7A44-450C-B389-D944A32FFCF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="167">
   <si>
     <t>ABESS RESULTS</t>
   </si>
@@ -127,9 +127,6 @@
     <t>0.8044 (0.1527)</t>
   </si>
   <si>
-    <t>0.7029 (0.2266)</t>
-  </si>
-  <si>
     <t>0.7900 (0.0745)</t>
   </si>
   <si>
@@ -268,9 +265,6 @@
     <t>0.77, 0.22</t>
   </si>
   <si>
-    <t>0.77, 0.08</t>
-  </si>
-  <si>
     <t>0.86, 0.52</t>
   </si>
   <si>
@@ -382,9 +376,6 @@
     <t>0.85, 0.57</t>
   </si>
   <si>
-    <t>0.72, 0.14</t>
-  </si>
-  <si>
     <t>0.81, 0.43</t>
   </si>
   <si>
@@ -530,6 +521,21 @@
   </si>
   <si>
     <t>Cox model results (HR, p-value)</t>
+  </si>
+  <si>
+    <t>0.69, 0.08</t>
+  </si>
+  <si>
+    <t>0.90, 0.64</t>
+  </si>
+  <si>
+    <t>0.68, 0.14</t>
+  </si>
+  <si>
+    <t>0.75, 0.32</t>
+  </si>
+  <si>
+    <t>0.6831 (0.2205)</t>
   </si>
 </sst>
 </file>
@@ -673,7 +679,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -691,36 +697,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -738,45 +732,38 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="37">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -1002,6 +989,14 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1105,6 +1100,14 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1119,80 +1122,80 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82CC2750-CD14-40AB-ABAD-70FA5D7EC4E8}" name="Tabla1" displayName="Tabla1" ref="A9:D16" totalsRowShown="0" headerRowDxfId="31" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82CC2750-CD14-40AB-ABAD-70FA5D7EC4E8}" name="Tabla1" displayName="Tabla1" ref="A9:D16" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A9:D16" xr:uid="{82CC2750-CD14-40AB-ABAD-70FA5D7EC4E8}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{993ECFB3-46BB-423B-8F2D-42C18AB267B0}" name="Time" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{F836BE5A-EE8A-4F0A-AEAC-77C43D6AAC33}" name="cg06785999" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{3216CD6C-3F26-40A8-870D-8FC4F4FBDEF4}" name="cg07095230" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{BDFAF975-8AA8-451D-BA0C-CDDFDBD06862}" name="cg00839579" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{993ECFB3-46BB-423B-8F2D-42C18AB267B0}" name="Time" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{F836BE5A-EE8A-4F0A-AEAC-77C43D6AAC33}" name="cg06785999" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{3216CD6C-3F26-40A8-870D-8FC4F4FBDEF4}" name="cg07095230" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{BDFAF975-8AA8-451D-BA0C-CDDFDBD06862}" name="cg00839579" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2BA47BF-FFDF-4D20-8C84-A49ACECB478E}" name="Tabla2" displayName="Tabla2" ref="G9:J16" totalsRowShown="0" headerRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2BA47BF-FFDF-4D20-8C84-A49ACECB478E}" name="Tabla2" displayName="Tabla2" ref="G9:J16" totalsRowShown="0" headerRowDxfId="30">
   <autoFilter ref="G9:J16" xr:uid="{C2BA47BF-FFDF-4D20-8C84-A49ACECB478E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D5F3E28B-B0B3-446E-A088-09E10A73893F}" name="Time" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{C141A2E1-5419-4DD7-919F-1D5A15F75FA1}" name="cg06785999" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{713BC794-ED09-406B-977E-7BA394E2E7EA}" name="cg07095230" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{CF55D58C-954B-4C41-8D99-D645811D560C}" name="cg00839579" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{D5F3E28B-B0B3-446E-A088-09E10A73893F}" name="Time" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{C141A2E1-5419-4DD7-919F-1D5A15F75FA1}" name="cg06785999" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{713BC794-ED09-406B-977E-7BA394E2E7EA}" name="cg07095230" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{CF55D58C-954B-4C41-8D99-D645811D560C}" name="cg00839579" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{67C75321-6869-45D5-A3CF-0E77AA37491A}" name="Tabla3" displayName="Tabla3" ref="A19:E26" totalsRowShown="0" headerRowDxfId="19" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{67C75321-6869-45D5-A3CF-0E77AA37491A}" name="Tabla3" displayName="Tabla3" ref="A19:E26" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="A19:E26" xr:uid="{67C75321-6869-45D5-A3CF-0E77AA37491A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{DF687A01-4DD6-4B1E-83ED-8E923B4D343D}" name="Time" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{E9E919BA-FAE6-44A3-B5F6-35EDB1B39571}" name="18q21.2" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{91138060-DBC0-45F4-B0B9-A7B4AA9E32FA}" name="21q11.2" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{DFB72076-0A68-44C0-89A0-F74334B2A3D9}" name="17p12" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{16701337-EBD6-4459-B117-7EA986EDB661}" name="9p21.3" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{DF687A01-4DD6-4B1E-83ED-8E923B4D343D}" name="Time" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{E9E919BA-FAE6-44A3-B5F6-35EDB1B39571}" name="18q21.2" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{91138060-DBC0-45F4-B0B9-A7B4AA9E32FA}" name="21q11.2" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{DFB72076-0A68-44C0-89A0-F74334B2A3D9}" name="17p12" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{16701337-EBD6-4459-B117-7EA986EDB661}" name="9p21.3" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{59D9BA3D-FC2B-4CA5-8A80-A1AFD29A57F6}" name="Tabla4" displayName="Tabla4" ref="G19:K26" totalsRowShown="0" headerRowDxfId="12" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{59D9BA3D-FC2B-4CA5-8A80-A1AFD29A57F6}" name="Tabla4" displayName="Tabla4" ref="G19:K26" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="G19:K26" xr:uid="{59D9BA3D-FC2B-4CA5-8A80-A1AFD29A57F6}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5ADE59F7-F9C6-4696-8F86-C65264C0A0EB}" name="Time" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{F1E8CACB-CA6B-4747-8867-836C367FEBBD}" name="18q21.2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{5CF9C49E-D9E4-4918-9BC1-5D2F4DDD74C2}" name="21q11.2" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{2B71EF22-D98B-49A4-924A-AEE8A306FE5D}" name="17p12" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{C830C0FF-9189-4573-9E3D-C69E0500EB5C}" name="9p21.3" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{5ADE59F7-F9C6-4696-8F86-C65264C0A0EB}" name="Time" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{F1E8CACB-CA6B-4747-8867-836C367FEBBD}" name="18q21.2" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{5CF9C49E-D9E4-4918-9BC1-5D2F4DDD74C2}" name="21q11.2" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{2B71EF22-D98B-49A4-924A-AEE8A306FE5D}" name="17p12" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{C830C0FF-9189-4573-9E3D-C69E0500EB5C}" name="9p21.3" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{FAB683BF-4D74-4A55-A976-B251557C24DA}" name="Tabla5" displayName="Tabla5" ref="A29:D36" totalsRowShown="0" headerRowDxfId="6" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{FAB683BF-4D74-4A55-A976-B251557C24DA}" name="Tabla5" displayName="Tabla5" ref="A29:D36" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A29:D36" xr:uid="{FAB683BF-4D74-4A55-A976-B251557C24DA}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{EA81F3F9-D114-4575-A02E-CAC3046ACCC2}" name="Time" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{C0C05769-5174-4025-8659-B99AD45AECEB}" name="cg06785999" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{5BBE3ED8-9C83-4A39-88EA-94F7CE7B9B52}" name="cg07095230" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{51D3D622-A488-451A-93AA-E6122159FC53}" name="cg00839579" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{EA81F3F9-D114-4575-A02E-CAC3046ACCC2}" name="Time" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{C0C05769-5174-4025-8659-B99AD45AECEB}" name="cg06785999" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{5BBE3ED8-9C83-4A39-88EA-94F7CE7B9B52}" name="cg07095230" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{51D3D622-A488-451A-93AA-E6122159FC53}" name="cg00839579" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5823CA53-63CA-47C8-8618-0C0AE8D2830C}" name="Tabla6" displayName="Tabla6" ref="G29:J36" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5823CA53-63CA-47C8-8618-0C0AE8D2830C}" name="Tabla6" displayName="Tabla6" ref="G29:J36" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="G29:J36" xr:uid="{5823CA53-63CA-47C8-8618-0C0AE8D2830C}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E43B94DA-4C4B-4A1F-9F49-33649B3F94C3}" name="Time" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{2A1C6E63-5A4A-4855-A11B-45D727C1AB98}" name="cg06785999" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{3ED2A264-7183-4926-8E77-A9EDFF048828}" name="cg07095230" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{9AB44483-CB4B-4346-B4E2-821659D480C8}" name="cg00839579" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E43B94DA-4C4B-4A1F-9F49-33649B3F94C3}" name="Time" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{2A1C6E63-5A4A-4855-A11B-45D727C1AB98}" name="cg06785999" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{3ED2A264-7183-4926-8E77-A9EDFF048828}" name="cg07095230" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{9AB44483-CB4B-4346-B4E2-821659D480C8}" name="cg00839579" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1536,7 +1539,7 @@
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -1564,15 +1567,15 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -1581,211 +1584,211 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="B9" s="12" t="s">
+      <c r="A9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="H9" s="12" t="s">
+      <c r="G9" t="s">
+        <v>160</v>
+      </c>
+      <c r="H9" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="J9" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="D10" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="G10" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="H10" s="12" t="s">
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" t="s">
+        <v>59</v>
+      </c>
+      <c r="I11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="J12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="J14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" t="s">
+        <v>56</v>
+      </c>
+      <c r="I16" t="s">
         <v>57</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="J16" t="s">
         <v>58</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="J11" s="14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="I12" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H13" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="I13" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="J13" s="14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H14" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="I14" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="J15" s="14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="I16" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
@@ -1794,472 +1797,472 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+      <c r="A19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" t="s">
+        <v>160</v>
+      </c>
+      <c r="H19" t="s">
+        <v>25</v>
+      </c>
+      <c r="I19" t="s">
+        <v>24</v>
+      </c>
+      <c r="J19" t="s">
+        <v>22</v>
+      </c>
+      <c r="K19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>162</v>
+      </c>
+      <c r="E20" t="s">
+        <v>76</v>
+      </c>
+      <c r="G20" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" t="s">
+        <v>100</v>
+      </c>
+      <c r="I20" t="s">
+        <v>101</v>
+      </c>
+      <c r="J20" t="s">
+        <v>102</v>
+      </c>
+      <c r="K20" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" t="s">
+        <v>80</v>
+      </c>
+      <c r="G21" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" t="s">
+        <v>104</v>
+      </c>
+      <c r="I21" t="s">
+        <v>105</v>
+      </c>
+      <c r="J21" t="s">
+        <v>106</v>
+      </c>
+      <c r="K21" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D22" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" t="s">
+        <v>9</v>
+      </c>
+      <c r="H22" t="s">
+        <v>108</v>
+      </c>
+      <c r="I22" t="s">
+        <v>109</v>
+      </c>
+      <c r="J22" t="s">
+        <v>110</v>
+      </c>
+      <c r="K22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E23" t="s">
+        <v>88</v>
+      </c>
+      <c r="G23" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" t="s">
+        <v>83</v>
+      </c>
+      <c r="I23" t="s">
+        <v>112</v>
+      </c>
+      <c r="J23" t="s">
+        <v>164</v>
+      </c>
+      <c r="K23" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" t="s">
+        <v>91</v>
+      </c>
+      <c r="E24" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" t="s">
+        <v>114</v>
+      </c>
+      <c r="I24" t="s">
+        <v>115</v>
+      </c>
+      <c r="J24" t="s">
+        <v>116</v>
+      </c>
+      <c r="K24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" t="s">
+        <v>95</v>
+      </c>
+      <c r="E25" t="s">
+        <v>96</v>
+      </c>
+      <c r="G25" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" t="s">
+        <v>118</v>
+      </c>
+      <c r="J25" t="s">
+        <v>119</v>
+      </c>
+      <c r="K25" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" t="s">
         <v>163</v>
       </c>
-      <c r="B19" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="I19" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="J19" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="K19" s="12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="H20" s="12" t="s">
+      <c r="G26" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" t="s">
+        <v>100</v>
+      </c>
+      <c r="I26" t="s">
+        <v>101</v>
+      </c>
+      <c r="J26" t="s">
         <v>102</v>
       </c>
-      <c r="I20" s="12" t="s">
+      <c r="K26" t="s">
         <v>103</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="K20" s="12" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="I21" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="J21" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="K21" s="12" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="I22" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="K22" s="12" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="I23" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="J23" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="K23" s="12" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="I24" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I25" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="J25" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="K25" s="12" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="I26" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="K26" s="12" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="B29" s="12" t="s">
+      <c r="A29" t="s">
+        <v>160</v>
+      </c>
+      <c r="B29" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" t="s">
         <v>16</v>
       </c>
-      <c r="G29" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="H29" s="12" t="s">
+      <c r="G29" t="s">
+        <v>160</v>
+      </c>
+      <c r="H29" t="s">
         <v>17</v>
       </c>
-      <c r="I29" s="12" t="s">
+      <c r="I29" t="s">
         <v>18</v>
       </c>
-      <c r="J29" s="12" t="s">
+      <c r="J29" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="A30" t="s">
         <v>7</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" t="s">
+        <v>121</v>
+      </c>
+      <c r="C30" t="s">
+        <v>122</v>
+      </c>
+      <c r="D30" t="s">
+        <v>123</v>
+      </c>
+      <c r="G30" t="s">
+        <v>7</v>
+      </c>
+      <c r="H30" t="s">
+        <v>142</v>
+      </c>
+      <c r="I30" t="s">
+        <v>143</v>
+      </c>
+      <c r="J30" s="10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" t="s">
         <v>124</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C31" t="s">
         <v>125</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="D31" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="G30" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="H30" s="12" t="s">
+      <c r="G31" t="s">
+        <v>8</v>
+      </c>
+      <c r="H31" t="s">
         <v>145</v>
       </c>
-      <c r="I30" s="12" t="s">
+      <c r="I31" t="s">
         <v>146</v>
       </c>
-      <c r="J30" s="14" t="s">
+      <c r="J31" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="12" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C32" t="s">
         <v>128</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D32" t="s">
         <v>129</v>
       </c>
-      <c r="G31" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H31" s="12" t="s">
+      <c r="G32" t="s">
+        <v>9</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="I31" s="12" t="s">
+      <c r="I32" t="s">
         <v>149</v>
       </c>
-      <c r="J31" s="12" t="s">
+      <c r="J32" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B32" s="14" t="s">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C33" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D33" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="G32" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H32" s="13" t="s">
+      <c r="G33" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="I32" s="12" t="s">
+      <c r="I33" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="J32" s="12" t="s">
+      <c r="J33" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B33" s="12" t="s">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" t="s">
         <v>133</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C34" t="s">
         <v>134</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D34" t="s">
         <v>135</v>
       </c>
-      <c r="G33" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H33" s="13" t="s">
+      <c r="G34" t="s">
+        <v>11</v>
+      </c>
+      <c r="H34" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="I33" s="13" t="s">
+      <c r="I34" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="J33" s="12" t="s">
+      <c r="J34" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34" s="12" t="s">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" t="s">
         <v>136</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C35" t="s">
         <v>137</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D35" t="s">
         <v>138</v>
       </c>
-      <c r="G34" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="H34" s="13" t="s">
+      <c r="G35" t="s">
+        <v>12</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="I34" s="13" t="s">
+      <c r="I35" t="s">
         <v>158</v>
       </c>
-      <c r="J34" s="12" t="s">
+      <c r="J35" s="10" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B35" s="12" t="s">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" t="s">
         <v>139</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C36" t="s">
         <v>140</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="D36" t="s">
         <v>141</v>
       </c>
-      <c r="G35" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="H35" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="I35" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="J35" s="14" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
+      <c r="G36" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="H36" t="s">
         <v>142</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="I36" t="s">
         <v>143</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="J36" s="10" t="s">
         <v>144</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="I36" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J36" s="14" t="s">
-        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2291,25 +2294,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D2" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="I2" s="10" t="s">
+      <c r="D2" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
+      <c r="E2" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="I2" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D3" s="11"/>
+      <c r="D3" s="30"/>
       <c r="E3" s="6" t="s">
         <v>17</v>
       </c>
@@ -2319,7 +2322,7 @@
       <c r="G3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="11"/>
+      <c r="I3" s="30"/>
       <c r="J3" s="6" t="s">
         <v>17</v>
       </c>
@@ -2334,263 +2337,237 @@
       <c r="D4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>126</v>
+      <c r="E4" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>123</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="28" t="s">
-        <v>145</v>
-      </c>
-      <c r="K4" s="28" t="s">
-        <v>146</v>
-      </c>
-      <c r="L4" s="29" t="s">
-        <v>147</v>
+      <c r="J4" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="K4" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="L4" s="23" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>129</v>
+      <c r="E5" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>126</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="K5" s="30" t="s">
-        <v>149</v>
-      </c>
-      <c r="L5" s="30" t="s">
-        <v>150</v>
+      <c r="J5" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="K5" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="L5" s="24" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="G6" s="26" t="s">
-        <v>132</v>
+      <c r="E6" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>129</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="K6" s="28" t="s">
-        <v>152</v>
-      </c>
-      <c r="L6" s="28" t="s">
-        <v>153</v>
+      <c r="J6" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="K6" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="L6" s="22" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="G7" s="25" t="s">
-        <v>135</v>
+      <c r="E7" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>132</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="L7" s="30" t="s">
-        <v>156</v>
+        <v>152</v>
+      </c>
+      <c r="L7" s="24" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="26" t="s">
-        <v>136</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="G8" s="26" t="s">
-        <v>138</v>
+      <c r="E8" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>135</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="31" t="s">
-        <v>157</v>
-      </c>
-      <c r="K8" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="L8" s="28" t="s">
-        <v>159</v>
+      <c r="J8" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="K8" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="L8" s="22" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="G9" s="24" t="s">
-        <v>141</v>
+      <c r="E9" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>138</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>12</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="K9" s="30" t="s">
-        <v>161</v>
+        <v>157</v>
+      </c>
+      <c r="K9" s="24" t="s">
+        <v>158</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>143</v>
-      </c>
-      <c r="G10" s="27" t="s">
-        <v>144</v>
+      <c r="E10" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>141</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J10" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="K10" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="L10" s="33" t="s">
-        <v>147</v>
+      <c r="J10" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="K10" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="L10" s="27" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="15"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
+      <c r="A12" s="3"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
+      <c r="A13" s="3"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="21"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="14"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="15"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
+      <c r="A15" s="3"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="C17" s="16"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.3">
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>